<commit_message>
DATN ho Ca Giay: Excel dieu tiet - doi ky hieu gach tren thanh 'tb', ghi chu cot k, w
- Q, V, Z, F co dau gach tren (ky tu to hop) lam Excel hien sai chi so duoi
  trong cung o (vd. '(Q +Q )/2'): doi thanh Qtb, Vtb, Ztb, Ftb o ca 3 file
- File dieu tiet lu: ghi chu (comment) o tieu de cot k, w; them vi du tra
  bang P1_KetVan gio 3 trong HuongDan
- So lieu khong doi (so sanh toan bo o so voi ban truoc: lech 0)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FZ7RkEfpZxiJWB6royQwfj
</commit_message>
<xml_diff>
--- a/DATN_HoCaGiay/TAI_VE/DieuTietLu_HaiTran_HoCaGiay.xlsx
+++ b/DATN_HoCaGiay/TAI_VE/DieuTietLu_HaiTran_HoCaGiay.xlsx
@@ -62,8 +62,160 @@
 </workbook>
 </file>
 
+<file path=xl/comments4.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <authors>
+    <author>Hướng dẫn</author>
+  </authors>
+  <commentList>
+    <comment ref="M15" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">k = MATCH(f₂; cột f của QuanHe; 1): số thứ tự dòng trong bảng QuanHe có f(k) ≤ f₂ &lt; f(k+1), tức Z₂ nằm giữa Z(k) và Z(k+1).
+Z(k) = 71,00 + (k − 1) × 0,10 m; ví dụ k = 38 → Z(k) = 74,70 m.
+Cột phụ để Excel tra bảng – không cần đưa vào thuyết minh.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="N15" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">w = [f₂ − f(k)] / [f(k+1) − f(k)]: f₂ nằm ở bao nhiêu phần quãng từ dòng k đến dòng k+1 (0 ÷ 1).
+Z₂, q tràn chính, q tràn sự cố, V₂ = giá trị dòng k + w × (dòng k+1 − dòng k).
+Cột phụ – không cần đưa vào thuyết minh.</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments5.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <authors>
+    <author>Hướng dẫn</author>
+  </authors>
+  <commentList>
+    <comment ref="M15" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">k = MATCH(f₂; cột f của QuanHe; 1): số thứ tự dòng trong bảng QuanHe có f(k) ≤ f₂ &lt; f(k+1), tức Z₂ nằm giữa Z(k) và Z(k+1).
+Z(k) = 71,00 + (k − 1) × 0,10 m; ví dụ k = 38 → Z(k) = 74,70 m.
+Cột phụ để Excel tra bảng – không cần đưa vào thuyết minh.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="N15" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">w = [f₂ − f(k)] / [f(k+1) − f(k)]: f₂ nằm ở bao nhiêu phần quãng từ dòng k đến dòng k+1 (0 ÷ 1).
+Z₂, q tràn chính, q tràn sự cố, V₂ = giá trị dòng k + w × (dòng k+1 − dòng k).
+Cột phụ – không cần đưa vào thuyết minh.</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments6.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <authors>
+    <author>Hướng dẫn</author>
+  </authors>
+  <commentList>
+    <comment ref="M15" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">k = MATCH(f₂; cột f của QuanHe; 1): số thứ tự dòng trong bảng QuanHe có f(k) ≤ f₂ &lt; f(k+1), tức Z₂ nằm giữa Z(k) và Z(k+1).
+Z(k) = 71,00 + (k − 1) × 0,10 m; ví dụ k = 38 → Z(k) = 74,70 m.
+Cột phụ để Excel tra bảng – không cần đưa vào thuyết minh.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="N15" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">w = [f₂ − f(k)] / [f(k+1) − f(k)]: f₂ nằm ở bao nhiêu phần quãng từ dòng k đến dòng k+1 (0 ÷ 1).
+Z₂, q tràn chính, q tràn sự cố, V₂ = giá trị dòng k + w × (dòng k+1 − dòng k).
+Cột phụ – không cần đưa vào thuyết minh.</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments7.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <authors>
+    <author>Hướng dẫn</author>
+  </authors>
+  <commentList>
+    <comment ref="M15" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">k = MATCH(f₂; cột f của QuanHe; 1): số thứ tự dòng trong bảng QuanHe có f(k) ≤ f₂ &lt; f(k+1), tức Z₂ nằm giữa Z(k) và Z(k+1).
+Z(k) = 71,00 + (k − 1) × 0,10 m; ví dụ k = 38 → Z(k) = 74,70 m.
+Cột phụ để Excel tra bảng – không cần đưa vào thuyết minh.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="N15" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">w = [f₂ − f(k)] / [f(k+1) − f(k)]: f₂ nằm ở bao nhiêu phần quãng từ dòng k đến dòng k+1 (0 ÷ 1).
+Z₂, q tràn chính, q tràn sự cố, V₂ = giá trị dòng k + w × (dòng k+1 − dòng k).
+Cột phụ – không cần đưa vào thuyết minh.</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="304" uniqueCount="177">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="178">
   <si>
     <t xml:space="preserve">ĐIỀU TIẾT LŨ HỒ CÀ GIÂY VỚI HAI TRÀN CÓ NGƯỠNG KHÁC NHAU – PHƯƠNG PHÁP PÔ-TA-PỐP</t>
   </si>
@@ -116,13 +268,16 @@
     <t xml:space="preserve">4. Phương pháp Pô-ta-pốp</t>
   </si>
   <si>
-    <t xml:space="preserve">(Q₁ + Q₂)/2·Δt − (q₁ + q₂)/2·Δt = V₂ − V₁    ⇒    V₂/Δt + q₂/2 = V₁/Δt + q₁/2 + Q̄ − q₁    ⇒    f₂ = f₁ + Q̄ − q₁</t>
+    <t xml:space="preserve">(Q₁ + Q₂)/2·Δt − (q₁ + q₂)/2·Δt = V₂ − V₁    ⇒    V₂/Δt + q₂/2 = V₁/Δt + q₁/2 + Qtb − q₁    ⇒    f₂ = f₁ + Qtb − q₁</t>
   </si>
   <si>
     <t xml:space="preserve">•  f = V/Δt + q/2 (đơn vị m³/s) chỉ phụ thuộc mực nước Z, nên lập sẵn bảng Z ~ V ~ q ~ f (sheet QuanHe, bước 0,1 m – thử bước 0,01 m kết quả chỉ lệch dưới 0,3 mm; một cột f cho trường hợp hai tràn, một cột cho trường hợp kẹt van).</t>
   </si>
   <si>
-    <t xml:space="preserve">•  Mỗi giờ: (1) Q̄ = (Q₁ + Q₂)/2; (2) f₂ = f₁ + Q̄ − q₁; (3) tra ngược bảng f ~ Z: tìm dòng k có f(k) ≤ f₂ &lt; f(k+1) (cột M, hàm MATCH) và tỷ lệ nội suy w = [f₂ − f(k)] / [f(k+1) − f(k)] (cột N); (4) Z₂, q tràn chính, q tràn sự cố, V₂ đều nội suy giữa dòng k và k+1 với CÙNG tỷ lệ w; (5) sang giờ sau với f₁ = f₂, q₁ = q₂.</t>
+    <t xml:space="preserve">•  Mỗi giờ: (1) Qtb = (Q₁ + Q₂)/2; (2) f₂ = f₁ + Qtb − q₁; (3) tra ngược bảng f ~ Z: tìm dòng k có f(k) ≤ f₂ &lt; f(k+1) (cột M, hàm MATCH) và tỷ lệ nội suy w = [f₂ − f(k)] / [f(k+1) − f(k)] (cột N); (4) Z₂, q tràn chính, q tràn sự cố, V₂ đều nội suy giữa dòng k và k+1 với CÙNG tỷ lệ w; (5) sang giờ sau với f₁ = f₂, q₁ = q₂.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">•  Ví dụ (sheet P1_KetVan, giờ 3, số liệu mặc định): f₂ = 10270,6 nằm giữa f(38) = 10114,4 (Z = 74,70 m) và f(39) = 10289,9 (Z = 74,80 m) → k = 38; w = (10270,6 − 10114,4)/(10289,9 − 10114,4) = 0,890 → Z₂ = 74,70 + 0,890 × 0,10 = 74,789 m; V₂ = 36,412 + 0,890 × (37,041 − 36,412) = 36,972·10⁶ m³.</t>
   </si>
   <si>
     <t xml:space="preserve">•  Vì sao dùng cùng w: khi đó V₂/Δt + q₂/2 đúng bằng f₂ (cột L) nên cân bằng nước khớp tuyệt đối. Nếu tính q₂ bằng công thức từ Z₂ còn f lại tra bảng thì hai bên lệch nhau một chút ở mỗi giờ, tích lũy thành sai số cân bằng nước.</t>
@@ -377,7 +532,7 @@
     <t xml:space="preserve">Cột f</t>
   </si>
   <si>
-    <t xml:space="preserve">Giờ 0: Z = MNDBT, q = q(MNDBT) theo trường hợp chọn. Từ giờ 1: f₂ = f₁ + Q̄ − q₁ → tìm dòng k, tỷ lệ w</t>
+    <t xml:space="preserve">Giờ 0: Z = MNDBT, q = q(MNDBT) theo trường hợp chọn. Từ giờ 1: f₂ = f₁ + Qtb − q₁ → tìm dòng k, tỷ lệ w</t>
   </si>
   <si>
     <t xml:space="preserve">Mực nước lớn nhất Zmax (m)</t>
@@ -407,7 +562,7 @@
     <t xml:space="preserve">Q đến (m³/s)</t>
   </si>
   <si>
-    <t xml:space="preserve">Q̄ = (Q₁+Q₂)/2</t>
+    <t xml:space="preserve">Qtb = (Q₁+Q₂)/2</t>
   </si>
   <si>
     <t xml:space="preserve">f₁ (giờ trước)</t>
@@ -416,7 +571,7 @@
     <t xml:space="preserve">q₁ (giờ trước)</t>
   </si>
   <si>
-    <t xml:space="preserve">f₂ = f₁ + Q̄ − q₁</t>
+    <t xml:space="preserve">f₂ = f₁ + Qtb − q₁</t>
   </si>
   <si>
     <t xml:space="preserve">Z₂ (m)</t>
@@ -608,7 +763,7 @@
     <numFmt numFmtId="168" formatCode="0.000"/>
     <numFmt numFmtId="169" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="17">
+  <fonts count="18">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -705,6 +860,11 @@
       <name val="Times New Roman"/>
       <family val="0"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b val="true"/>
@@ -2302,11 +2462,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="18174793"/>
-        <c:axId val="23430601"/>
+        <c:axId val="61349872"/>
+        <c:axId val="14030336"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="18174793"/>
+        <c:axId val="61349872"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2372,7 +2532,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="23430601"/>
+        <c:crossAx val="14030336"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2380,7 +2540,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="23430601"/>
+        <c:axId val="14030336"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1000"/>
@@ -2458,7 +2618,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="18174793"/>
+        <c:crossAx val="61349872"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="100"/>
@@ -4073,11 +4233,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="89839813"/>
-        <c:axId val="54148851"/>
+        <c:axId val="4485176"/>
+        <c:axId val="34296797"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="89839813"/>
+        <c:axId val="4485176"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4143,7 +4303,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="54148851"/>
+        <c:crossAx val="34296797"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -4151,7 +4311,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="54148851"/>
+        <c:axId val="34296797"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="80"/>
@@ -4229,7 +4389,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="89839813"/>
+        <c:crossAx val="4485176"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="1"/>
@@ -4963,7 +5123,7 @@
     <tabColor rgb="FFA65A10"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="B1:B31"/>
+  <dimension ref="B1:B32"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="3"/>
@@ -5070,28 +5230,28 @@
         <v>19</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="46.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B21" s="4" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B22" s="4" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B23" s="4" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B24" s="3" t="s">
+    <row r="24" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B24" s="4" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B25" s="4" t="s">
+    <row r="25" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B25" s="3" t="s">
         <v>24</v>
       </c>
     </row>
@@ -5100,12 +5260,12 @@
         <v>25</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B27" s="4" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="28" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B28" s="4" t="s">
         <v>27</v>
       </c>
@@ -5115,14 +5275,19 @@
         <v>28</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B30" s="3" t="s">
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B30" s="4" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B31" s="4" t="s">
+    <row r="31" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B31" s="3" t="s">
         <v>30</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B32" s="4" t="s">
+        <v>31</v>
       </c>
     </row>
   </sheetData>
@@ -5154,31 +5319,31 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="6" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="9" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E5" s="9"/>
       <c r="F5" s="9"/>
@@ -5187,16 +5352,16 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B6" s="11" t="n">
         <v>74.7</v>
       </c>
       <c r="C6" s="12" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E6" s="13"/>
       <c r="F6" s="13"/>
@@ -5205,16 +5370,16 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B7" s="14" t="n">
         <v>1</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E7" s="13"/>
       <c r="F7" s="13"/>
@@ -5223,14 +5388,14 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B8" s="14" t="n">
         <f aca="false">dt_h*3600</f>
         <v>3600</v>
       </c>
       <c r="C8" s="12" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D8" s="13"/>
       <c r="E8" s="13"/>
@@ -5240,13 +5405,13 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="10" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B9" s="15" t="n">
         <v>9.81</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D9" s="13"/>
       <c r="E9" s="13"/>
@@ -5256,21 +5421,21 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="8" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="9" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E12" s="9"/>
       <c r="F12" s="9"/>
@@ -5279,16 +5444,16 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="10" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B13" s="11" t="n">
         <v>74.7</v>
       </c>
       <c r="C13" s="12" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D13" s="13" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E13" s="13"/>
       <c r="F13" s="13"/>
@@ -5297,16 +5462,16 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="10" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B14" s="16" t="n">
         <v>9</v>
       </c>
       <c r="C14" s="12" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D14" s="13" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E14" s="13"/>
       <c r="F14" s="13"/>
@@ -5315,16 +5480,16 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="10" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B15" s="11" t="n">
         <v>2.4</v>
       </c>
       <c r="C15" s="12" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D15" s="13" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E15" s="13"/>
       <c r="F15" s="13"/>
@@ -5333,14 +5498,14 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="10" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B16" s="11" t="n">
         <v>0.45</v>
       </c>
       <c r="C16" s="12"/>
       <c r="D16" s="13" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E16" s="13"/>
       <c r="F16" s="13"/>
@@ -5349,14 +5514,14 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="10" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B17" s="11" t="n">
         <v>0.7</v>
       </c>
       <c r="C17" s="12"/>
       <c r="D17" s="13" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E17" s="13"/>
       <c r="F17" s="13"/>
@@ -5365,14 +5530,14 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="10" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B18" s="11" t="n">
         <v>0.45</v>
       </c>
       <c r="C18" s="12"/>
       <c r="D18" s="13" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="E18" s="13"/>
       <c r="F18" s="13"/>
@@ -5381,14 +5546,14 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="10" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B19" s="11" t="n">
         <v>1</v>
       </c>
       <c r="C19" s="12"/>
       <c r="D19" s="13" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E19" s="13"/>
       <c r="F19" s="13"/>
@@ -5397,21 +5562,21 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="8" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="9" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C22" s="9" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D22" s="9" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E22" s="9"/>
       <c r="F22" s="9"/>
@@ -5420,16 +5585,16 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="10" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B23" s="11" t="n">
         <v>71</v>
       </c>
       <c r="C23" s="12" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D23" s="13" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E23" s="13"/>
       <c r="F23" s="13"/>
@@ -5438,13 +5603,13 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="10" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B24" s="16" t="n">
         <v>1</v>
       </c>
       <c r="C24" s="12" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D24" s="13"/>
       <c r="E24" s="13"/>
@@ -5454,16 +5619,16 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="10" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B25" s="11" t="n">
         <v>5</v>
       </c>
       <c r="C25" s="12" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D25" s="13" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E25" s="13"/>
       <c r="F25" s="13"/>
@@ -5472,14 +5637,14 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="10" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B26" s="11" t="n">
         <v>0.45</v>
       </c>
       <c r="C26" s="12"/>
       <c r="D26" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E26" s="13"/>
       <c r="F26" s="13"/>
@@ -5488,7 +5653,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="10" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B27" s="11" t="n">
         <v>0.7</v>
@@ -5502,14 +5667,14 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="10" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B28" s="11" t="n">
         <v>0.45</v>
       </c>
       <c r="C28" s="12"/>
       <c r="D28" s="13" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E28" s="13"/>
       <c r="F28" s="13"/>
@@ -5518,14 +5683,14 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="10" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B29" s="11" t="n">
         <v>1</v>
       </c>
       <c r="C29" s="12"/>
       <c r="D29" s="13" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E29" s="13"/>
       <c r="F29" s="13"/>
@@ -5534,12 +5699,12 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="8" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="17" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B32" s="18" t="n">
         <v>1</v>
@@ -5550,13 +5715,13 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="9" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B33" s="9" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C33" s="9" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5570,7 +5735,7 @@
         <v>4</v>
       </c>
       <c r="D34" s="7" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5584,10 +5749,10 @@
         <v>4</v>
       </c>
       <c r="E35" s="9" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="F35" s="9" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5601,7 +5766,7 @@
         <v>84</v>
       </c>
       <c r="D36" s="20" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E36" s="21" t="n">
         <f aca="false">SUMPRODUCT((B34:B69+B35:B70)/2)*dt_s/1000000+B70/2*dt_s/1000000</f>
@@ -5623,7 +5788,7 @@
         <v>324</v>
       </c>
       <c r="D37" s="20" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E37" s="22" t="n">
         <v>32.43</v>
@@ -5643,7 +5808,7 @@
         <v>652</v>
       </c>
       <c r="D38" s="7" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6000,21 +6165,21 @@
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="8" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="9" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B74" s="9" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C74" s="9" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D74" s="9" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6028,7 +6193,7 @@
         <v>0</v>
       </c>
       <c r="D75" s="7" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6398,53 +6563,53 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="6" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="I4" s="9" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="J4" s="9" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="K4" s="9" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="L4" s="9" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="M4" s="9" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11933,32 +12098,32 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="6" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="10" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B3" s="10"/>
       <c r="C3" s="33" t="n">
         <v>1</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E3" s="10"/>
       <c r="F3" s="34" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="G3" s="34"/>
       <c r="H3" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="13" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B4" s="13"/>
       <c r="C4" s="35" t="n">
@@ -11966,7 +12131,7 @@
         <v>1</v>
       </c>
       <c r="D4" s="13" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E4" s="13"/>
       <c r="F4" s="35" t="n">
@@ -11976,12 +12141,12 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H5" s="7" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B6" s="10"/>
       <c r="C6" s="10"/>
@@ -11992,12 +12157,12 @@
         <v>77.6079256047331</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B7" s="10"/>
       <c r="C7" s="10"/>
@@ -12010,7 +12175,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B8" s="10"/>
       <c r="C8" s="10"/>
@@ -12023,7 +12188,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="10" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B9" s="10"/>
       <c r="C9" s="10"/>
@@ -12040,7 +12205,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="10" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B10" s="10"/>
       <c r="C10" s="10"/>
@@ -12057,7 +12222,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="10" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B11" s="10"/>
       <c r="C11" s="10"/>
@@ -12070,7 +12235,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="10" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B12" s="10"/>
       <c r="C12" s="10"/>
@@ -12083,46 +12248,46 @@
     </row>
     <row r="15" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="9" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C15" s="9" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D15" s="9" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F15" s="9" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G15" s="9" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H15" s="9" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="I15" s="9" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="J15" s="9" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="K15" s="9" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="L15" s="9" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="M15" s="9" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="N15" s="9" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14943,6 +15108,7 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -14968,32 +15134,32 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="6" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="10" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B3" s="10"/>
       <c r="C3" s="33" t="n">
         <v>1</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E3" s="10"/>
       <c r="F3" s="34" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="G3" s="34"/>
       <c r="H3" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="13" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B4" s="13"/>
       <c r="C4" s="35" t="n">
@@ -15001,7 +15167,7 @@
         <v>1</v>
       </c>
       <c r="D4" s="13" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E4" s="13"/>
       <c r="F4" s="35" t="n">
@@ -15011,12 +15177,12 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H5" s="7" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B6" s="10"/>
       <c r="C6" s="10"/>
@@ -15027,12 +15193,12 @@
         <v>78.2048023895375</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B7" s="10"/>
       <c r="C7" s="10"/>
@@ -15045,7 +15211,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B8" s="10"/>
       <c r="C8" s="10"/>
@@ -15058,7 +15224,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="10" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B9" s="10"/>
       <c r="C9" s="10"/>
@@ -15075,7 +15241,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="10" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B10" s="10"/>
       <c r="C10" s="10"/>
@@ -15092,7 +15258,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="10" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B11" s="10"/>
       <c r="C11" s="10"/>
@@ -15105,7 +15271,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="10" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B12" s="10"/>
       <c r="C12" s="10"/>
@@ -15118,46 +15284,46 @@
     </row>
     <row r="15" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="9" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C15" s="9" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D15" s="9" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F15" s="9" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G15" s="9" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H15" s="9" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="I15" s="9" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="J15" s="9" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="K15" s="9" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="L15" s="9" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="M15" s="9" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="N15" s="9" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17978,6 +18144,7 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -18003,32 +18170,32 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="6" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="10" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B3" s="10"/>
       <c r="C3" s="33" t="n">
         <v>0.2</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E3" s="10"/>
       <c r="F3" s="34" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="G3" s="34"/>
       <c r="H3" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="13" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B4" s="13"/>
       <c r="C4" s="35" t="n">
@@ -18036,7 +18203,7 @@
         <v>2</v>
       </c>
       <c r="D4" s="13" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E4" s="13"/>
       <c r="F4" s="35" t="n">
@@ -18046,12 +18213,12 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H5" s="7" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B6" s="10"/>
       <c r="C6" s="10"/>
@@ -18062,12 +18229,12 @@
         <v>78.5143600647203</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B7" s="10"/>
       <c r="C7" s="10"/>
@@ -18080,7 +18247,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B8" s="10"/>
       <c r="C8" s="10"/>
@@ -18093,7 +18260,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="10" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B9" s="10"/>
       <c r="C9" s="10"/>
@@ -18110,7 +18277,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="10" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B10" s="10"/>
       <c r="C10" s="10"/>
@@ -18127,7 +18294,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="10" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B11" s="10"/>
       <c r="C11" s="10"/>
@@ -18140,7 +18307,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="10" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B12" s="10"/>
       <c r="C12" s="10"/>
@@ -18153,46 +18320,46 @@
     </row>
     <row r="15" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="9" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C15" s="9" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D15" s="9" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F15" s="9" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G15" s="9" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H15" s="9" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="I15" s="9" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="J15" s="9" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="K15" s="9" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="L15" s="9" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="M15" s="9" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="N15" s="9" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21013,6 +21180,7 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -21038,32 +21206,32 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="6" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="10" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B3" s="10"/>
       <c r="C3" s="33" t="n">
         <v>0.2</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E3" s="10"/>
       <c r="F3" s="34" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="G3" s="34"/>
       <c r="H3" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="13" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B4" s="13"/>
       <c r="C4" s="35" t="n">
@@ -21071,7 +21239,7 @@
         <v>2</v>
       </c>
       <c r="D4" s="13" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E4" s="13"/>
       <c r="F4" s="35" t="n">
@@ -21081,12 +21249,12 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H5" s="7" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B6" s="10"/>
       <c r="C6" s="10"/>
@@ -21097,12 +21265,12 @@
         <v>79.1402507451014</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B7" s="10"/>
       <c r="C7" s="10"/>
@@ -21115,7 +21283,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B8" s="10"/>
       <c r="C8" s="10"/>
@@ -21128,7 +21296,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="10" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B9" s="10"/>
       <c r="C9" s="10"/>
@@ -21145,7 +21313,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="10" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B10" s="10"/>
       <c r="C10" s="10"/>
@@ -21162,7 +21330,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="10" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B11" s="10"/>
       <c r="C11" s="10"/>
@@ -21175,7 +21343,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="10" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B12" s="10"/>
       <c r="C12" s="10"/>
@@ -21188,46 +21356,46 @@
     </row>
     <row r="15" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="9" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C15" s="9" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D15" s="9" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F15" s="9" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G15" s="9" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H15" s="9" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="I15" s="9" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="J15" s="9" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="K15" s="9" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="L15" s="9" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="M15" s="9" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="N15" s="9" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -24048,6 +24216,7 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -24072,31 +24241,31 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="6" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B4" s="10"/>
       <c r="C4" s="11" t="n">
         <v>74.7</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="E4" s="10"/>
       <c r="F4" s="11" t="n">
         <v>79.5</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="H4" s="10"/>
       <c r="I4" s="33" t="n">
@@ -24105,40 +24274,40 @@
     </row>
     <row r="6" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="9" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C6" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="D6" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="E6" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="F6" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="G6" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="H6" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="I6" s="9" t="s">
         <v>87</v>
       </c>
-      <c r="D6" s="9" t="s">
-        <v>89</v>
-      </c>
-      <c r="E6" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="F6" s="9" t="s">
-        <v>92</v>
-      </c>
-      <c r="G6" s="9" t="s">
-        <v>93</v>
-      </c>
-      <c r="H6" s="9" t="s">
-        <v>80</v>
-      </c>
-      <c r="I6" s="9" t="s">
-        <v>86</v>
-      </c>
       <c r="J6" s="9" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="K6" s="9" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="L6" s="9" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29239,44 +29408,44 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="6" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="9" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="F3" s="9" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="G3" s="9" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="H3" s="9" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="I3" s="9" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="J3" s="9" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B4" s="12" t="str">
         <f aca="false">P1_HaiTran!C3&amp;" – "&amp;P1_HaiTran!F3</f>
@@ -29310,12 +29479,12 @@
         <v>77.63</v>
       </c>
       <c r="J4" s="13" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B5" s="12" t="str">
         <f aca="false">P1_KetVan!C3&amp;" – "&amp;P1_KetVan!F3</f>
@@ -29349,12 +29518,12 @@
         <v>78.21</v>
       </c>
       <c r="J5" s="13" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B6" s="12" t="str">
         <f aca="false">P02_HaiTran!C3&amp;" – "&amp;P02_HaiTran!F3</f>
@@ -29388,12 +29557,12 @@
         <v>78.54</v>
       </c>
       <c r="J6" s="13" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B7" s="12" t="str">
         <f aca="false">P02_KetVan!C3&amp;" – "&amp;P02_KetVan!F3</f>
@@ -29427,38 +29596,38 @@
         <v>79.14</v>
       </c>
       <c r="J7" s="13" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="8" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="9" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D12" s="9"/>
       <c r="E12" s="9"/>
       <c r="F12" s="9" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="G12" s="9"/>
       <c r="H12" s="9"/>
@@ -29467,7 +29636,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="10" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B13" s="22" t="n">
         <v>78.28</v>
@@ -29476,7 +29645,7 @@
         <v>79.15</v>
       </c>
       <c r="F13" s="13" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="G13" s="13"/>
       <c r="H13" s="13"/>
@@ -29485,7 +29654,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="10" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B14" s="22" t="n">
         <v>78.37</v>
@@ -29494,7 +29663,7 @@
         <v>79.39</v>
       </c>
       <c r="F14" s="13" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="G14" s="13"/>
       <c r="H14" s="13"/>
@@ -29503,7 +29672,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="10" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="B15" s="21" t="n">
         <f aca="false">C5</f>
@@ -29514,7 +29683,7 @@
         <v>79.1402507451014</v>
       </c>
       <c r="F15" s="13" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="G15" s="13"/>
       <c r="H15" s="13"/>
@@ -29523,7 +29692,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="10" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B16" s="21" t="n">
         <f aca="false">C4</f>
@@ -29534,7 +29703,7 @@
         <v>78.5143600647203</v>
       </c>
       <c r="F16" s="13" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="G16" s="13"/>
       <c r="H16" s="13"/>
@@ -29543,7 +29712,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="20" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D18" s="21" t="n">
         <f aca="false">C4</f>
@@ -29552,7 +29721,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="20" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="D19" s="21" t="n">
         <f aca="false">C6</f>
@@ -29561,33 +29730,33 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="8" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="9" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C22" s="9" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="D22" s="9" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="E22" s="9" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="F22" s="9" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="G22" s="9" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="H22" s="9" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>